<commit_message>
added win pct code and html to index
</commit_message>
<xml_diff>
--- a/TeamFriends_History.xlsx
+++ b/TeamFriends_History.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Sites\TeamFriendsFantasy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E00547-6836-4E12-916B-3C76446DC85C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B123BD0-A986-46A0-B697-486E12ACAD14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="677" firstSheet="1" activeTab="18" xr2:uid="{960D14EB-F112-4860-840A-1E6B67EAFFB3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="677" firstSheet="1" activeTab="19" xr2:uid="{960D14EB-F112-4860-840A-1E6B67EAFFB3}"/>
   </bookViews>
   <sheets>
     <sheet name="2005" sheetId="16" r:id="rId1"/>
@@ -1211,20 +1211,14 @@
     <xf numFmtId="9" fontId="0" fillId="8" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="11" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="10" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1232,19 +1226,25 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1723,7 +1723,7 @@
         <v>2248.5</v>
       </c>
       <c r="K3" s="60"/>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="58" t="s">
         <v>166</v>
       </c>
     </row>
@@ -1756,10 +1756,10 @@
       <c r="I4" s="1">
         <v>2325.5</v>
       </c>
-      <c r="K4" s="59" t="s">
+      <c r="K4" s="58" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="59"/>
+      <c r="L4" s="58"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1790,7 +1790,7 @@
       <c r="I5" s="1">
         <v>2430.5</v>
       </c>
-      <c r="K5" s="59"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B6">
@@ -1848,24 +1848,24 @@
       <c r="I7">
         <v>1856</v>
       </c>
-      <c r="K7" s="58" t="s">
+      <c r="K7" s="64" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="K8" s="58"/>
-      <c r="L8" s="58" t="s">
+      <c r="K8" s="64"/>
+      <c r="L8" s="64" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="58" t="s">
         <v>168</v>
       </c>
-      <c r="L9" s="58"/>
+      <c r="L9" s="64"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="K10" s="59"/>
+      <c r="K10" s="58"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L12" s="6" t="s">
@@ -1873,7 +1873,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="L13" s="58" t="s">
+      <c r="L13" s="64" t="s">
         <v>169</v>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       <c r="D14" t="s">
         <v>180</v>
       </c>
-      <c r="L14" s="58"/>
+      <c r="L14" s="64"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1905,7 +1905,7 @@
       <c r="D15">
         <v>0</v>
       </c>
-      <c r="L15" s="59" t="s">
+      <c r="L15" s="58" t="s">
         <v>164</v>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       <c r="B16" t="s">
         <v>182</v>
       </c>
-      <c r="L16" s="59"/>
+      <c r="L16" s="58"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -2346,7 +2346,7 @@
       <c r="J3" s="1">
         <v>1670.76</v>
       </c>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="58" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       <c r="J4" s="1">
         <v>1595.7</v>
       </c>
-      <c r="L4" s="66"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2455,7 +2455,7 @@
         <v>1622.42</v>
       </c>
       <c r="L6" s="60"/>
-      <c r="N6" s="62" t="s">
+      <c r="N6" s="63" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2488,7 +2488,7 @@
       <c r="J7">
         <v>1329.76</v>
       </c>
-      <c r="N7" s="67"/>
+      <c r="N7" s="66"/>
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -2521,7 +2521,7 @@
       <c r="J8" s="10">
         <v>1426.34</v>
       </c>
-      <c r="N8" s="63" t="s">
+      <c r="N8" s="61" t="s">
         <v>96</v>
       </c>
       <c r="P8" s="14"/>
@@ -2530,10 +2530,10 @@
       <c r="A9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="59" t="s">
+      <c r="L9" s="58" t="s">
         <v>96</v>
       </c>
-      <c r="N9" s="63"/>
+      <c r="N9" s="61"/>
       <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -2567,7 +2567,7 @@
       <c r="J10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L10" s="66"/>
+      <c r="L10" s="59"/>
       <c r="M10" s="10"/>
       <c r="N10" s="14"/>
       <c r="P10" s="14"/>
@@ -2604,7 +2604,7 @@
       <c r="J11" s="1">
         <v>1668.7</v>
       </c>
-      <c r="L11" s="58" t="s">
+      <c r="L11" s="64" t="s">
         <v>88</v>
       </c>
       <c r="P11" s="14"/>
@@ -2641,8 +2641,8 @@
       <c r="J12" s="1">
         <v>1621.08</v>
       </c>
-      <c r="L12" s="58"/>
-      <c r="P12" s="63" t="s">
+      <c r="L12" s="64"/>
+      <c r="P12" s="61" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2675,7 +2675,7 @@
       <c r="J13">
         <v>1604.78</v>
       </c>
-      <c r="P13" s="64"/>
+      <c r="P13" s="62"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B14">
@@ -2706,7 +2706,7 @@
       <c r="J14">
         <v>1563.12</v>
       </c>
-      <c r="P14" s="62" t="s">
+      <c r="P14" s="63" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2739,10 +2739,10 @@
       <c r="J15">
         <v>1437.26</v>
       </c>
-      <c r="L15" s="59" t="s">
+      <c r="L15" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="P15" s="62"/>
+      <c r="P15" s="63"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B16">
@@ -2773,12 +2773,12 @@
       <c r="J16">
         <v>1463.6</v>
       </c>
-      <c r="L16" s="66"/>
+      <c r="L16" s="59"/>
       <c r="M16" s="10"/>
       <c r="P16" s="14"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L17" s="58" t="s">
+      <c r="L17" s="64" t="s">
         <v>60</v>
       </c>
       <c r="N17" s="14"/>
@@ -2786,20 +2786,20 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="L18" s="58"/>
-      <c r="N18" s="62" t="s">
+      <c r="L18" s="64"/>
+      <c r="N18" s="63" t="s">
         <v>73</v>
       </c>
       <c r="P18" s="14"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="N19" s="67"/>
+      <c r="N19" s="66"/>
       <c r="O19" s="10"/>
       <c r="P19" s="14"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N20" s="63" t="s">
+      <c r="N20" s="61" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2813,10 +2813,10 @@
       <c r="F21" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="L21" s="59" t="s">
+      <c r="L21" s="58" t="s">
         <v>101</v>
       </c>
-      <c r="N21" s="63"/>
+      <c r="N21" s="61"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -2831,7 +2831,7 @@
       <c r="F22" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="L22" s="66"/>
+      <c r="L22" s="59"/>
       <c r="M22" s="10"/>
       <c r="N22" s="14"/>
     </row>
@@ -2845,7 +2845,7 @@
       <c r="F23" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="L23" s="58" t="s">
+      <c r="L23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2859,7 +2859,7 @@
       <c r="F24" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="L24" s="58"/>
+      <c r="L24" s="64"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -2874,7 +2874,7 @@
       <c r="A26" t="s">
         <v>30</v>
       </c>
-      <c r="P26" s="58" t="s">
+      <c r="P26" s="64" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="P28" s="59" t="s">
+      <c r="P28" s="58" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2896,18 +2896,13 @@
       <c r="A29" t="s">
         <v>49</v>
       </c>
-      <c r="P29" s="59"/>
+      <c r="P29" s="58"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C3:J8">
     <sortCondition descending="1" ref="H3:H8"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="L9:L10"/>
     <mergeCell ref="L23:L24"/>
     <mergeCell ref="P26:P27"/>
     <mergeCell ref="P28:P29"/>
@@ -2919,6 +2914,11 @@
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="L21:L22"/>
     <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="L9:L10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3019,7 +3019,7 @@
       <c r="J3" s="1">
         <v>1593.46</v>
       </c>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="58" t="s">
         <v>96</v>
       </c>
     </row>
@@ -3055,7 +3055,7 @@
       <c r="J4" s="1">
         <v>1541.96</v>
       </c>
-      <c r="L4" s="66"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3125,7 +3125,7 @@
         <v>1471.44</v>
       </c>
       <c r="L6" s="60"/>
-      <c r="N6" s="63" t="s">
+      <c r="N6" s="61" t="s">
         <v>96</v>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
       <c r="J7">
         <v>1396.52</v>
       </c>
-      <c r="N7" s="64"/>
+      <c r="N7" s="62"/>
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -3191,7 +3191,7 @@
       <c r="J8" s="10">
         <v>1071.8599999999999</v>
       </c>
-      <c r="N8" s="62" t="s">
+      <c r="N8" s="63" t="s">
         <v>60</v>
       </c>
       <c r="P8" s="14"/>
@@ -3200,10 +3200,10 @@
       <c r="A9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="58" t="s">
+      <c r="L9" s="64" t="s">
         <v>99</v>
       </c>
-      <c r="N9" s="62"/>
+      <c r="N9" s="63"/>
       <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -3274,7 +3274,7 @@
       <c r="J11" s="1">
         <v>1662.04</v>
       </c>
-      <c r="L11" s="59" t="s">
+      <c r="L11" s="58" t="s">
         <v>60</v>
       </c>
       <c r="P11" s="14"/>
@@ -3311,8 +3311,8 @@
       <c r="J12" s="1">
         <v>1508.68</v>
       </c>
-      <c r="L12" s="59"/>
-      <c r="P12" s="63" t="s">
+      <c r="L12" s="58"/>
+      <c r="P12" s="61" t="s">
         <v>96</v>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
       <c r="J13" s="1">
         <v>1559.22</v>
       </c>
-      <c r="P13" s="64"/>
+      <c r="P13" s="62"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B14">
@@ -3379,7 +3379,7 @@
       <c r="J14">
         <v>1534.62</v>
       </c>
-      <c r="P14" s="62" t="s">
+      <c r="P14" s="63" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3412,10 +3412,10 @@
       <c r="J15">
         <v>1411.74</v>
       </c>
-      <c r="L15" s="59" t="s">
+      <c r="L15" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="P15" s="62"/>
+      <c r="P15" s="63"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B16">
@@ -3446,12 +3446,12 @@
       <c r="J16">
         <v>1163.0999999999999</v>
       </c>
-      <c r="L16" s="66"/>
+      <c r="L16" s="59"/>
       <c r="M16" s="10"/>
       <c r="P16" s="14"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L17" s="58" t="s">
+      <c r="L17" s="64" t="s">
         <v>119</v>
       </c>
       <c r="N17" s="14"/>
@@ -3459,20 +3459,20 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="L18" s="58"/>
-      <c r="N18" s="62" t="s">
+      <c r="L18" s="64"/>
+      <c r="N18" s="63" t="s">
         <v>73</v>
       </c>
       <c r="P18" s="14"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="N19" s="67"/>
+      <c r="N19" s="66"/>
       <c r="O19" s="10"/>
       <c r="P19" s="14"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N20" s="63" t="s">
+      <c r="N20" s="61" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3486,10 +3486,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="L21" s="59" t="s">
+      <c r="L21" s="58" t="s">
         <v>115</v>
       </c>
-      <c r="N21" s="63"/>
+      <c r="N21" s="61"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -3504,7 +3504,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="L22" s="66"/>
+      <c r="L22" s="59"/>
       <c r="M22" s="10"/>
       <c r="N22" s="14"/>
     </row>
@@ -3518,7 +3518,7 @@
       <c r="F23" s="16">
         <v>40</v>
       </c>
-      <c r="L23" s="58" t="s">
+      <c r="L23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="L24" s="58"/>
+      <c r="L24" s="64"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -3559,7 +3559,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="P26" s="58" t="s">
+      <c r="P26" s="64" t="s">
         <v>60</v>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="P28" s="59" t="s">
+      <c r="P28" s="58" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3581,18 +3581,13 @@
       <c r="A29" t="s">
         <v>49</v>
       </c>
-      <c r="P29" s="59"/>
+      <c r="P29" s="58"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C11:J16">
     <sortCondition descending="1" ref="H11:H16"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="L9:L10"/>
     <mergeCell ref="L23:L24"/>
     <mergeCell ref="P26:P27"/>
     <mergeCell ref="P28:P29"/>
@@ -3604,6 +3599,11 @@
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="L21:L22"/>
     <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="L9:L10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3704,7 +3704,7 @@
       <c r="J3" s="1">
         <v>1792.26</v>
       </c>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="58" t="s">
         <v>123</v>
       </c>
     </row>
@@ -3740,7 +3740,7 @@
       <c r="J4" s="1">
         <v>1746.74</v>
       </c>
-      <c r="L4" s="66"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3807,7 +3807,7 @@
         <v>1608.62</v>
       </c>
       <c r="L6" s="60"/>
-      <c r="N6" s="62" t="s">
+      <c r="N6" s="63" t="s">
         <v>123</v>
       </c>
     </row>
@@ -3840,7 +3840,7 @@
       <c r="J7">
         <v>1608.1</v>
       </c>
-      <c r="N7" s="67"/>
+      <c r="N7" s="66"/>
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -3873,7 +3873,7 @@
       <c r="J8" s="10">
         <v>1419.32</v>
       </c>
-      <c r="N8" s="63" t="s">
+      <c r="N8" s="61" t="s">
         <v>116</v>
       </c>
       <c r="P8" s="14"/>
@@ -3882,10 +3882,10 @@
       <c r="A9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="59" t="s">
+      <c r="L9" s="58" t="s">
         <v>116</v>
       </c>
-      <c r="N9" s="63"/>
+      <c r="N9" s="61"/>
       <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -3919,7 +3919,7 @@
       <c r="J10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L10" s="66"/>
+      <c r="L10" s="59"/>
       <c r="M10" s="10"/>
       <c r="N10" s="14"/>
       <c r="P10" s="14"/>
@@ -3956,7 +3956,7 @@
       <c r="J11" s="1">
         <v>1895.72</v>
       </c>
-      <c r="L11" s="58" t="s">
+      <c r="L11" s="64" t="s">
         <v>124</v>
       </c>
       <c r="P11" s="14"/>
@@ -3993,8 +3993,8 @@
       <c r="J12" s="1">
         <v>1666.54</v>
       </c>
-      <c r="L12" s="58"/>
-      <c r="P12" s="62" t="s">
+      <c r="L12" s="64"/>
+      <c r="P12" s="63" t="s">
         <v>116</v>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       <c r="J13" s="1">
         <v>1770.32</v>
       </c>
-      <c r="P13" s="67"/>
+      <c r="P13" s="66"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -4064,7 +4064,7 @@
       <c r="J14" s="1">
         <v>1642.38</v>
       </c>
-      <c r="P14" s="63" t="s">
+      <c r="P14" s="61" t="s">
         <v>122</v>
       </c>
     </row>
@@ -4097,10 +4097,10 @@
       <c r="J15">
         <v>1496.7</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="L15" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="P15" s="63"/>
+      <c r="P15" s="61"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B16">
@@ -4136,7 +4136,7 @@
       <c r="P16" s="14"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L17" s="59" t="s">
+      <c r="L17" s="58" t="s">
         <v>122</v>
       </c>
       <c r="N17" s="14"/>
@@ -4144,20 +4144,20 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="L18" s="59"/>
-      <c r="N18" s="63" t="s">
+      <c r="L18" s="58"/>
+      <c r="N18" s="61" t="s">
         <v>122</v>
       </c>
       <c r="P18" s="14"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="N19" s="64"/>
+      <c r="N19" s="62"/>
       <c r="O19" s="10"/>
       <c r="P19" s="14"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N20" s="62" t="s">
+      <c r="N20" s="63" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4171,10 +4171,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="L21" s="59" t="s">
+      <c r="L21" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="N21" s="62"/>
+      <c r="N21" s="63"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -4189,7 +4189,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="L22" s="66"/>
+      <c r="L22" s="59"/>
       <c r="M22" s="10"/>
       <c r="N22" s="14"/>
     </row>
@@ -4203,7 +4203,7 @@
       <c r="F23" s="16">
         <v>40</v>
       </c>
-      <c r="L23" s="58" t="s">
+      <c r="L23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -4217,7 +4217,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="L24" s="58"/>
+      <c r="L24" s="64"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -4244,7 +4244,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="P26" s="59" t="s">
+      <c r="P26" s="58" t="s">
         <v>123</v>
       </c>
     </row>
@@ -4252,13 +4252,13 @@
       <c r="A27" t="s">
         <v>83</v>
       </c>
-      <c r="P27" s="66"/>
+      <c r="P27" s="59"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="P28" s="58" t="s">
+      <c r="P28" s="64" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4266,18 +4266,13 @@
       <c r="A29" t="s">
         <v>49</v>
       </c>
-      <c r="P29" s="58"/>
+      <c r="P29" s="64"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C11:J16">
     <sortCondition descending="1" ref="H11:H16"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="L9:L10"/>
     <mergeCell ref="L23:L24"/>
     <mergeCell ref="P26:P27"/>
     <mergeCell ref="P28:P29"/>
@@ -4289,6 +4284,11 @@
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="L21:L22"/>
     <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="L9:L10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4389,7 +4389,7 @@
       <c r="J3" s="1">
         <v>1530.24</v>
       </c>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="58" t="s">
         <v>137</v>
       </c>
     </row>
@@ -4425,7 +4425,7 @@
       <c r="J4" s="1">
         <v>1530.84</v>
       </c>
-      <c r="L4" s="66"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4492,7 +4492,7 @@
         <v>1541.3</v>
       </c>
       <c r="L6" s="60"/>
-      <c r="N6" s="62" t="s">
+      <c r="N6" s="63" t="s">
         <v>124</v>
       </c>
     </row>
@@ -4525,7 +4525,7 @@
       <c r="J7">
         <v>1631.78</v>
       </c>
-      <c r="N7" s="67"/>
+      <c r="N7" s="66"/>
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -4558,7 +4558,7 @@
       <c r="J8" s="10">
         <v>1453.8</v>
       </c>
-      <c r="N8" s="63" t="s">
+      <c r="N8" s="61" t="s">
         <v>60</v>
       </c>
       <c r="P8" s="14"/>
@@ -4567,10 +4567,10 @@
       <c r="A9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="58" t="s">
+      <c r="L9" s="64" t="s">
         <v>136</v>
       </c>
-      <c r="N9" s="63"/>
+      <c r="N9" s="61"/>
       <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -4641,7 +4641,7 @@
       <c r="J11" s="1">
         <v>1851.34</v>
       </c>
-      <c r="L11" s="59" t="s">
+      <c r="L11" s="58" t="s">
         <v>60</v>
       </c>
       <c r="P11" s="14"/>
@@ -4678,8 +4678,8 @@
       <c r="J12" s="1">
         <v>1742.32</v>
       </c>
-      <c r="L12" s="59"/>
-      <c r="P12" s="63" t="s">
+      <c r="L12" s="58"/>
+      <c r="P12" s="61" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4715,7 +4715,7 @@
       <c r="J13" s="1">
         <v>1566.5</v>
       </c>
-      <c r="P13" s="64"/>
+      <c r="P13" s="62"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -4749,7 +4749,7 @@
       <c r="J14" s="1">
         <v>1453.92</v>
       </c>
-      <c r="P14" s="62" t="s">
+      <c r="P14" s="63" t="s">
         <v>122</v>
       </c>
     </row>
@@ -4782,10 +4782,10 @@
       <c r="J15">
         <v>1573</v>
       </c>
-      <c r="L15" s="59" t="s">
+      <c r="L15" s="58" t="s">
         <v>134</v>
       </c>
-      <c r="P15" s="62"/>
+      <c r="P15" s="63"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B16">
@@ -4816,12 +4816,12 @@
       <c r="J16">
         <v>1656.98</v>
       </c>
-      <c r="L16" s="66"/>
+      <c r="L16" s="59"/>
       <c r="M16" s="10"/>
       <c r="P16" s="14"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L17" s="58" t="s">
+      <c r="L17" s="64" t="s">
         <v>135</v>
       </c>
       <c r="N17" s="14"/>
@@ -4829,20 +4829,20 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="L18" s="58"/>
-      <c r="N18" s="63" t="s">
+      <c r="L18" s="64"/>
+      <c r="N18" s="61" t="s">
         <v>134</v>
       </c>
       <c r="P18" s="14"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="N19" s="64"/>
+      <c r="N19" s="62"/>
       <c r="O19" s="10"/>
       <c r="P19" s="14"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N20" s="62" t="s">
+      <c r="N20" s="63" t="s">
         <v>96</v>
       </c>
     </row>
@@ -4856,10 +4856,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="L21" s="59" t="s">
+      <c r="L21" s="58" t="s">
         <v>96</v>
       </c>
-      <c r="N21" s="62"/>
+      <c r="N21" s="63"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -4874,7 +4874,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="L22" s="66"/>
+      <c r="L22" s="59"/>
       <c r="M22" s="10"/>
       <c r="N22" s="14"/>
     </row>
@@ -4888,7 +4888,7 @@
       <c r="F23" s="16">
         <v>40</v>
       </c>
-      <c r="L23" s="58" t="s">
+      <c r="L23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="L24" s="58"/>
+      <c r="L24" s="64"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -4929,7 +4929,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="P26" s="58" t="s">
+      <c r="P26" s="64" t="s">
         <v>124</v>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="P28" s="59" t="s">
+      <c r="P28" s="58" t="s">
         <v>96</v>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       <c r="A29" t="s">
         <v>49</v>
       </c>
-      <c r="P29" s="59"/>
+      <c r="P29" s="58"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
@@ -4963,11 +4963,6 @@
     <sortCondition descending="1" ref="H11:H16"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="L9:L10"/>
     <mergeCell ref="L23:L24"/>
     <mergeCell ref="P26:P27"/>
     <mergeCell ref="P28:P29"/>
@@ -4979,6 +4974,11 @@
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="L21:L22"/>
     <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="L9:L10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5079,7 +5079,7 @@
       <c r="J3" s="1">
         <v>1744.88</v>
       </c>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="58" t="s">
         <v>135</v>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       <c r="J4" s="1">
         <v>1652.44</v>
       </c>
-      <c r="L4" s="66"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5185,7 +5185,7 @@
         <v>1612.58</v>
       </c>
       <c r="L6" s="60"/>
-      <c r="N6" s="63" t="s">
+      <c r="N6" s="61" t="s">
         <v>135</v>
       </c>
     </row>
@@ -5218,7 +5218,7 @@
       <c r="J7">
         <v>1567.06</v>
       </c>
-      <c r="N7" s="64"/>
+      <c r="N7" s="62"/>
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
       <c r="J8" s="10">
         <v>1467.82</v>
       </c>
-      <c r="N8" s="62" t="s">
+      <c r="N8" s="63" t="s">
         <v>141</v>
       </c>
       <c r="P8" s="14"/>
@@ -5260,10 +5260,10 @@
       <c r="A9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="58" t="s">
+      <c r="L9" s="64" t="s">
         <v>142</v>
       </c>
-      <c r="N9" s="62"/>
+      <c r="N9" s="63"/>
       <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -5334,7 +5334,7 @@
       <c r="J11" s="1">
         <v>1764.64</v>
       </c>
-      <c r="L11" s="59" t="s">
+      <c r="L11" s="58" t="s">
         <v>141</v>
       </c>
       <c r="P11" s="14"/>
@@ -5371,8 +5371,8 @@
       <c r="J12" s="1">
         <v>1574.5</v>
       </c>
-      <c r="L12" s="59"/>
-      <c r="P12" s="62" t="s">
+      <c r="L12" s="58"/>
+      <c r="P12" s="63" t="s">
         <v>135</v>
       </c>
     </row>
@@ -5408,7 +5408,7 @@
       <c r="J13" s="1">
         <v>1644.76</v>
       </c>
-      <c r="P13" s="67"/>
+      <c r="P13" s="66"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B14">
@@ -5439,7 +5439,7 @@
       <c r="J14">
         <v>1397.72</v>
       </c>
-      <c r="P14" s="63" t="s">
+      <c r="P14" s="61" t="s">
         <v>118</v>
       </c>
     </row>
@@ -5472,10 +5472,10 @@
       <c r="J15">
         <v>1368.44</v>
       </c>
-      <c r="L15" s="59" t="s">
+      <c r="L15" s="58" t="s">
         <v>118</v>
       </c>
-      <c r="P15" s="63"/>
+      <c r="P15" s="61"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B16">
@@ -5506,12 +5506,12 @@
       <c r="J16">
         <v>1319.8</v>
       </c>
-      <c r="L16" s="66"/>
+      <c r="L16" s="59"/>
       <c r="M16" s="10"/>
       <c r="P16" s="14"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L17" s="58" t="s">
+      <c r="L17" s="64" t="s">
         <v>96</v>
       </c>
       <c r="N17" s="14"/>
@@ -5519,20 +5519,20 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="L18" s="58"/>
-      <c r="N18" s="63" t="s">
+      <c r="L18" s="64"/>
+      <c r="N18" s="61" t="s">
         <v>118</v>
       </c>
       <c r="P18" s="14"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="N19" s="64"/>
+      <c r="N19" s="62"/>
       <c r="O19" s="10"/>
       <c r="P19" s="14"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N20" s="62" t="s">
+      <c r="N20" s="63" t="s">
         <v>115</v>
       </c>
     </row>
@@ -5546,10 +5546,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="L21" s="59" t="s">
+      <c r="L21" s="58" t="s">
         <v>115</v>
       </c>
-      <c r="N21" s="62"/>
+      <c r="N21" s="63"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
@@ -5564,7 +5564,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="L22" s="66"/>
+      <c r="L22" s="59"/>
       <c r="M22" s="10"/>
       <c r="N22" s="14"/>
     </row>
@@ -5579,7 +5579,7 @@
       <c r="F23" s="16">
         <v>40</v>
       </c>
-      <c r="L23" s="58" t="s">
+      <c r="L23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -5594,7 +5594,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="L24" s="58"/>
+      <c r="L24" s="64"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -5623,7 +5623,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="P26" s="58" t="s">
+      <c r="P26" s="64" t="s">
         <v>141</v>
       </c>
     </row>
@@ -5639,7 +5639,7 @@
         <v>32</v>
       </c>
       <c r="B28" s="5"/>
-      <c r="P28" s="59" t="s">
+      <c r="P28" s="58" t="s">
         <v>115</v>
       </c>
     </row>
@@ -5648,7 +5648,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="P29" s="59"/>
+      <c r="P29" s="58"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
@@ -5661,11 +5661,6 @@
     <sortCondition descending="1" ref="H11:H16"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="L9:L10"/>
     <mergeCell ref="L23:L24"/>
     <mergeCell ref="P26:P27"/>
     <mergeCell ref="P28:P29"/>
@@ -5677,6 +5672,11 @@
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="L21:L22"/>
     <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="L9:L10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5795,7 +5795,7 @@
       <c r="I3" s="1">
         <v>1830.48</v>
       </c>
-      <c r="K3" s="59" t="s">
+      <c r="K3" s="58" t="s">
         <v>146</v>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
       <c r="I4" s="1">
         <v>1957.51</v>
       </c>
-      <c r="K4" s="66"/>
+      <c r="K4" s="59"/>
       <c r="L4" s="10"/>
     </row>
     <row r="5" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5895,7 +5895,7 @@
         <v>1810.54</v>
       </c>
       <c r="K6" s="60"/>
-      <c r="M6" s="62" t="s">
+      <c r="M6" s="63" t="s">
         <v>146</v>
       </c>
     </row>
@@ -5928,7 +5928,7 @@
       <c r="I7" s="1">
         <v>1739.8</v>
       </c>
-      <c r="M7" s="67"/>
+      <c r="M7" s="66"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -5957,7 +5957,7 @@
       <c r="I8">
         <v>1557.34</v>
       </c>
-      <c r="M8" s="63" t="s">
+      <c r="M8" s="61" t="s">
         <v>115</v>
       </c>
       <c r="O8" s="14"/>
@@ -5988,10 +5988,10 @@
       <c r="I9">
         <v>1632.8</v>
       </c>
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="58" t="s">
         <v>115</v>
       </c>
-      <c r="M9" s="63"/>
+      <c r="M9" s="61"/>
       <c r="O9" s="14"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -6020,7 +6020,7 @@
       <c r="I10">
         <v>1479.68</v>
       </c>
-      <c r="K10" s="66"/>
+      <c r="K10" s="59"/>
       <c r="L10" s="10"/>
       <c r="M10" s="14"/>
       <c r="O10" s="14"/>
@@ -6051,7 +6051,7 @@
       <c r="I11">
         <v>1326.38</v>
       </c>
-      <c r="K11" s="58" t="s">
+      <c r="K11" s="64" t="s">
         <v>135</v>
       </c>
       <c r="O11" s="14"/>
@@ -6082,8 +6082,8 @@
       <c r="I12">
         <v>1491.86</v>
       </c>
-      <c r="K12" s="58"/>
-      <c r="O12" s="63" t="s">
+      <c r="K12" s="64"/>
+      <c r="O12" s="61" t="s">
         <v>115</v>
       </c>
     </row>
@@ -6113,29 +6113,29 @@
       <c r="I13">
         <v>1391.5</v>
       </c>
-      <c r="O13" s="64"/>
+      <c r="O13" s="62"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H14" s="4"/>
-      <c r="O14" s="62" t="s">
+      <c r="O14" s="63" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H15" s="4"/>
-      <c r="K15" s="59" t="s">
+      <c r="K15" s="58" t="s">
         <v>144</v>
       </c>
-      <c r="O15" s="62"/>
+      <c r="O15" s="63"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H16" s="4"/>
-      <c r="K16" s="66"/>
+      <c r="K16" s="59"/>
       <c r="L16" s="10"/>
       <c r="O16" s="14"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K17" s="58" t="s">
+      <c r="K17" s="64" t="s">
         <v>99</v>
       </c>
       <c r="M17" s="14"/>
@@ -6143,20 +6143,20 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="K18" s="58"/>
-      <c r="M18" s="63" t="s">
+      <c r="K18" s="64"/>
+      <c r="M18" s="61" t="s">
         <v>144</v>
       </c>
       <c r="O18" s="14"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="M19" s="64"/>
+      <c r="M19" s="62"/>
       <c r="N19" s="10"/>
       <c r="O19" s="14"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M20" s="68" t="s">
+      <c r="M20" s="69" t="s">
         <v>153</v>
       </c>
     </row>
@@ -6170,10 +6170,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="K21" s="59" t="s">
+      <c r="K21" s="58" t="s">
         <v>153</v>
       </c>
-      <c r="M21" s="62"/>
+      <c r="M21" s="63"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
@@ -6188,7 +6188,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="K22" s="66"/>
+      <c r="K22" s="59"/>
       <c r="L22" s="10"/>
       <c r="M22" s="14"/>
     </row>
@@ -6203,7 +6203,7 @@
       <c r="F23" s="17">
         <v>30</v>
       </c>
-      <c r="K23" s="58" t="s">
+      <c r="K23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="K24" s="58"/>
+      <c r="K24" s="64"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -6247,7 +6247,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="O26" s="58" t="s">
+      <c r="O26" s="64" t="s">
         <v>146</v>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
         <v>32</v>
       </c>
       <c r="B28" s="5"/>
-      <c r="O28" s="59" t="s">
+      <c r="O28" s="58" t="s">
         <v>153</v>
       </c>
     </row>
@@ -6272,7 +6272,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="O29" s="59"/>
+      <c r="O29" s="58"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
@@ -6285,11 +6285,6 @@
     <sortCondition descending="1" ref="H2:H13"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="K9:K10"/>
     <mergeCell ref="K23:K24"/>
     <mergeCell ref="O26:O27"/>
     <mergeCell ref="O28:O29"/>
@@ -6301,6 +6296,11 @@
     <mergeCell ref="M20:M21"/>
     <mergeCell ref="K21:K22"/>
     <mergeCell ref="K11:K12"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="K9:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6419,7 +6419,7 @@
       <c r="I3" s="1">
         <v>1668.12</v>
       </c>
-      <c r="K3" s="59" t="s">
+      <c r="K3" s="58" t="s">
         <v>151</v>
       </c>
     </row>
@@ -6452,7 +6452,7 @@
       <c r="I4" s="1">
         <v>1799.34</v>
       </c>
-      <c r="K4" s="66"/>
+      <c r="K4" s="59"/>
       <c r="L4" s="10"/>
     </row>
     <row r="5" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -6519,7 +6519,7 @@
         <v>1688.86</v>
       </c>
       <c r="K6" s="60"/>
-      <c r="M6" s="62" t="s">
+      <c r="M6" s="63" t="s">
         <v>151</v>
       </c>
     </row>
@@ -6552,7 +6552,7 @@
       <c r="I7" s="1">
         <v>1626.76</v>
       </c>
-      <c r="M7" s="67"/>
+      <c r="M7" s="66"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -6581,7 +6581,7 @@
       <c r="I8">
         <v>1557.08</v>
       </c>
-      <c r="M8" s="63" t="s">
+      <c r="M8" s="61" t="s">
         <v>145</v>
       </c>
       <c r="O8" s="14"/>
@@ -6612,10 +6612,10 @@
       <c r="I9">
         <v>1554.84</v>
       </c>
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="58" t="s">
         <v>153</v>
       </c>
-      <c r="M9" s="63"/>
+      <c r="M9" s="61"/>
       <c r="O9" s="14"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -6644,7 +6644,7 @@
       <c r="I10">
         <v>1463.02</v>
       </c>
-      <c r="K10" s="66"/>
+      <c r="K10" s="59"/>
       <c r="L10" s="10"/>
       <c r="M10" s="14"/>
       <c r="O10" s="14"/>
@@ -6675,7 +6675,7 @@
       <c r="I11">
         <v>1798.06</v>
       </c>
-      <c r="K11" s="58" t="s">
+      <c r="K11" s="64" t="s">
         <v>118</v>
       </c>
       <c r="O11" s="14"/>
@@ -6706,8 +6706,8 @@
       <c r="I12">
         <v>1635.74</v>
       </c>
-      <c r="K12" s="58"/>
-      <c r="O12" s="63" t="s">
+      <c r="K12" s="64"/>
+      <c r="O12" s="61" t="s">
         <v>153</v>
       </c>
     </row>
@@ -6737,20 +6737,20 @@
       <c r="I13">
         <v>1620.5</v>
       </c>
-      <c r="O13" s="64"/>
+      <c r="O13" s="62"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H14" s="4"/>
-      <c r="O14" s="62" t="s">
+      <c r="O14" s="63" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H15" s="4"/>
-      <c r="K15" s="58" t="s">
+      <c r="K15" s="64" t="s">
         <v>144</v>
       </c>
-      <c r="O15" s="62"/>
+      <c r="O15" s="63"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H16" s="4"/>
@@ -6759,7 +6759,7 @@
       <c r="O16" s="14"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K17" s="59" t="s">
+      <c r="K17" s="58" t="s">
         <v>60</v>
       </c>
       <c r="M17" s="14"/>
@@ -6767,20 +6767,20 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="K18" s="59"/>
-      <c r="M18" s="62" t="s">
+      <c r="K18" s="58"/>
+      <c r="M18" s="63" t="s">
         <v>60</v>
       </c>
       <c r="O18" s="14"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="M19" s="67"/>
+      <c r="M19" s="66"/>
       <c r="N19" s="10"/>
       <c r="O19" s="14"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M20" s="69" t="s">
+      <c r="M20" s="67" t="s">
         <v>150</v>
       </c>
     </row>
@@ -6794,10 +6794,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="K21" s="59" t="s">
+      <c r="K21" s="58" t="s">
         <v>150</v>
       </c>
-      <c r="M21" s="63"/>
+      <c r="M21" s="61"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
@@ -6812,7 +6812,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="K22" s="66"/>
+      <c r="K22" s="59"/>
       <c r="L22" s="10"/>
       <c r="M22" s="14"/>
     </row>
@@ -6827,7 +6827,7 @@
       <c r="F23" s="16">
         <v>30</v>
       </c>
-      <c r="K23" s="58" t="s">
+      <c r="K23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -6842,7 +6842,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="K24" s="58"/>
+      <c r="K24" s="64"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -6871,7 +6871,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="O26" s="59" t="s">
+      <c r="O26" s="58" t="s">
         <v>151</v>
       </c>
     </row>
@@ -6880,7 +6880,7 @@
         <v>83</v>
       </c>
       <c r="B27" s="5"/>
-      <c r="O27" s="66"/>
+      <c r="O27" s="59"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
@@ -6890,7 +6890,7 @@
       <c r="C28" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="O28" s="58" t="s">
+      <c r="O28" s="64" t="s">
         <v>60</v>
       </c>
     </row>
@@ -6899,7 +6899,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="O29" s="58"/>
+      <c r="O29" s="64"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
@@ -6912,11 +6912,6 @@
     <sortCondition descending="1" ref="H2:H13"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="K9:K10"/>
     <mergeCell ref="K23:K24"/>
     <mergeCell ref="O26:O27"/>
     <mergeCell ref="O28:O29"/>
@@ -6928,6 +6923,11 @@
     <mergeCell ref="M20:M21"/>
     <mergeCell ref="K21:K22"/>
     <mergeCell ref="K11:K12"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="K9:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7046,7 +7046,7 @@
       <c r="I3" s="1">
         <v>1879.82</v>
       </c>
-      <c r="K3" s="59" t="s">
+      <c r="K3" s="58" t="s">
         <v>154</v>
       </c>
     </row>
@@ -7079,7 +7079,7 @@
       <c r="I4" s="1">
         <v>1689.34</v>
       </c>
-      <c r="K4" s="66"/>
+      <c r="K4" s="59"/>
       <c r="L4" s="10"/>
     </row>
     <row r="5" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7146,7 +7146,7 @@
         <v>1695.94</v>
       </c>
       <c r="K6" s="60"/>
-      <c r="M6" s="63" t="s">
+      <c r="M6" s="61" t="s">
         <v>154</v>
       </c>
     </row>
@@ -7179,7 +7179,7 @@
       <c r="I7" s="1">
         <v>1633.82</v>
       </c>
-      <c r="M7" s="64"/>
+      <c r="M7" s="62"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -7208,7 +7208,7 @@
       <c r="I8">
         <v>1591.5</v>
       </c>
-      <c r="M8" s="62" t="s">
+      <c r="M8" s="63" t="s">
         <v>146</v>
       </c>
       <c r="O8" s="14"/>
@@ -7239,10 +7239,10 @@
       <c r="I9">
         <v>1566.6</v>
       </c>
-      <c r="K9" s="58" t="s">
+      <c r="K9" s="64" t="s">
         <v>155</v>
       </c>
-      <c r="M9" s="62"/>
+      <c r="M9" s="63"/>
       <c r="O9" s="14"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -7302,7 +7302,7 @@
       <c r="I11">
         <v>1740</v>
       </c>
-      <c r="K11" s="59" t="s">
+      <c r="K11" s="58" t="s">
         <v>146</v>
       </c>
       <c r="O11" s="14"/>
@@ -7333,8 +7333,8 @@
       <c r="I12">
         <v>1435.98</v>
       </c>
-      <c r="K12" s="59"/>
-      <c r="O12" s="62" t="s">
+      <c r="K12" s="58"/>
+      <c r="O12" s="63" t="s">
         <v>154</v>
       </c>
     </row>
@@ -7364,29 +7364,29 @@
       <c r="I13">
         <v>1443.12</v>
       </c>
-      <c r="O13" s="67"/>
+      <c r="O13" s="66"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H14" s="4"/>
-      <c r="O14" s="63" t="s">
+      <c r="O14" s="61" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H15" s="4"/>
-      <c r="K15" s="59" t="s">
+      <c r="K15" s="58" t="s">
         <v>144</v>
       </c>
-      <c r="O15" s="63"/>
+      <c r="O15" s="61"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H16" s="4"/>
-      <c r="K16" s="66"/>
+      <c r="K16" s="59"/>
       <c r="L16" s="10"/>
       <c r="O16" s="14"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K17" s="58" t="s">
+      <c r="K17" s="64" t="s">
         <v>147</v>
       </c>
       <c r="M17" s="14"/>
@@ -7394,20 +7394,20 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="K18" s="58"/>
-      <c r="M18" s="62" t="s">
+      <c r="K18" s="64"/>
+      <c r="M18" s="63" t="s">
         <v>144</v>
       </c>
       <c r="O18" s="14"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="M19" s="67"/>
+      <c r="M19" s="66"/>
       <c r="N19" s="10"/>
       <c r="O19" s="14"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M20" s="69" t="s">
+      <c r="M20" s="67" t="s">
         <v>136</v>
       </c>
     </row>
@@ -7421,10 +7421,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="K21" s="59" t="s">
+      <c r="K21" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="M21" s="63"/>
+      <c r="M21" s="61"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
@@ -7439,7 +7439,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="K22" s="66"/>
+      <c r="K22" s="59"/>
       <c r="L22" s="10"/>
       <c r="M22" s="14"/>
     </row>
@@ -7454,7 +7454,7 @@
       <c r="F23" s="16">
         <v>30</v>
       </c>
-      <c r="K23" s="58" t="s">
+      <c r="K23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -7469,7 +7469,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="K24" s="58"/>
+      <c r="K24" s="64"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -7498,7 +7498,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="O26" s="59" t="s">
+      <c r="O26" s="58" t="s">
         <v>146</v>
       </c>
     </row>
@@ -7507,7 +7507,7 @@
         <v>83</v>
       </c>
       <c r="B27" s="5"/>
-      <c r="O27" s="66"/>
+      <c r="O27" s="59"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
@@ -7517,7 +7517,7 @@
       <c r="C28" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="O28" s="58" t="s">
+      <c r="O28" s="64" t="s">
         <v>144</v>
       </c>
     </row>
@@ -7526,7 +7526,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="O29" s="58"/>
+      <c r="O29" s="64"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
@@ -7539,11 +7539,6 @@
     <sortCondition descending="1" ref="H2:H13"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="K9:K10"/>
     <mergeCell ref="K23:K24"/>
     <mergeCell ref="O26:O27"/>
     <mergeCell ref="O28:O29"/>
@@ -7555,6 +7550,11 @@
     <mergeCell ref="M20:M21"/>
     <mergeCell ref="K21:K22"/>
     <mergeCell ref="K11:K12"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="K9:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7673,7 +7673,7 @@
       <c r="I3" s="1">
         <v>1810.84</v>
       </c>
-      <c r="K3" s="59" t="s">
+      <c r="K3" s="58" t="s">
         <v>146</v>
       </c>
     </row>
@@ -7706,7 +7706,7 @@
       <c r="I4" s="1">
         <v>1781.88</v>
       </c>
-      <c r="K4" s="66"/>
+      <c r="K4" s="59"/>
       <c r="L4" s="10"/>
     </row>
     <row r="5" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7773,7 +7773,7 @@
         <v>1712.9</v>
       </c>
       <c r="K6" s="60"/>
-      <c r="M6" s="63" t="s">
+      <c r="M6" s="61" t="s">
         <v>146</v>
       </c>
     </row>
@@ -7806,7 +7806,7 @@
       <c r="I7" s="1">
         <v>1821.42</v>
       </c>
-      <c r="M7" s="64"/>
+      <c r="M7" s="62"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -7835,7 +7835,7 @@
       <c r="I8">
         <v>1771.9</v>
       </c>
-      <c r="M8" s="62" t="s">
+      <c r="M8" s="63" t="s">
         <v>275</v>
       </c>
       <c r="O8" s="14"/>
@@ -7866,10 +7866,10 @@
       <c r="I9">
         <v>1582.7</v>
       </c>
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="58" t="s">
         <v>275</v>
       </c>
-      <c r="M9" s="62"/>
+      <c r="M9" s="63"/>
       <c r="O9" s="14"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -7898,7 +7898,7 @@
       <c r="I10">
         <v>1709.36</v>
       </c>
-      <c r="K10" s="66"/>
+      <c r="K10" s="59"/>
       <c r="L10" s="10"/>
       <c r="M10" s="14"/>
       <c r="O10" s="14"/>
@@ -7929,7 +7929,7 @@
       <c r="I11">
         <v>1628.92</v>
       </c>
-      <c r="K11" s="58" t="s">
+      <c r="K11" s="64" t="s">
         <v>60</v>
       </c>
       <c r="O11" s="14"/>
@@ -7960,8 +7960,8 @@
       <c r="I12">
         <v>1418.44</v>
       </c>
-      <c r="K12" s="58"/>
-      <c r="O12" s="63" t="s">
+      <c r="K12" s="64"/>
+      <c r="O12" s="61" t="s">
         <v>146</v>
       </c>
     </row>
@@ -7991,29 +7991,29 @@
       <c r="I13">
         <v>1315.52</v>
       </c>
-      <c r="O13" s="64"/>
+      <c r="O13" s="62"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H14" s="4"/>
-      <c r="O14" s="68" t="s">
+      <c r="O14" s="69" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H15" s="4"/>
-      <c r="K15" s="59" t="s">
+      <c r="K15" s="58" t="s">
         <v>144</v>
       </c>
-      <c r="O15" s="62"/>
+      <c r="O15" s="63"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H16" s="4"/>
-      <c r="K16" s="66"/>
+      <c r="K16" s="59"/>
       <c r="L16" s="10"/>
       <c r="O16" s="14"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K17" s="58" t="s">
+      <c r="K17" s="64" t="s">
         <v>154</v>
       </c>
       <c r="M17" s="14"/>
@@ -8021,20 +8021,20 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="K18" s="58"/>
-      <c r="M18" s="62" t="s">
+      <c r="K18" s="64"/>
+      <c r="M18" s="63" t="s">
         <v>144</v>
       </c>
       <c r="O18" s="14"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="M19" s="67"/>
+      <c r="M19" s="66"/>
       <c r="N19" s="10"/>
       <c r="O19" s="14"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M20" s="69" t="s">
+      <c r="M20" s="67" t="s">
         <v>272</v>
       </c>
     </row>
@@ -8048,10 +8048,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="K21" s="59" t="s">
+      <c r="K21" s="58" t="s">
         <v>272</v>
       </c>
-      <c r="M21" s="63"/>
+      <c r="M21" s="61"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
@@ -8066,7 +8066,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="K22" s="66"/>
+      <c r="K22" s="59"/>
       <c r="L22" s="10"/>
       <c r="M22" s="14"/>
     </row>
@@ -8081,7 +8081,7 @@
       <c r="F23" s="16">
         <v>30</v>
       </c>
-      <c r="K23" s="58" t="s">
+      <c r="K23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -8096,7 +8096,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="K24" s="58"/>
+      <c r="K24" s="64"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -8125,7 +8125,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="O26" s="59" t="s">
+      <c r="O26" s="58" t="s">
         <v>144</v>
       </c>
     </row>
@@ -8134,7 +8134,7 @@
         <v>83</v>
       </c>
       <c r="B27" s="5"/>
-      <c r="O27" s="66"/>
+      <c r="O27" s="59"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
@@ -8144,7 +8144,7 @@
       <c r="C28" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="O28" s="58" t="s">
+      <c r="O28" s="64" t="s">
         <v>275</v>
       </c>
     </row>
@@ -8153,7 +8153,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="O29" s="58"/>
+      <c r="O29" s="64"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
@@ -8163,11 +8163,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="K9:K10"/>
     <mergeCell ref="K23:K24"/>
     <mergeCell ref="O26:O27"/>
     <mergeCell ref="O28:O29"/>
@@ -8179,6 +8174,11 @@
     <mergeCell ref="M20:M21"/>
     <mergeCell ref="K21:K22"/>
     <mergeCell ref="K11:K12"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="K9:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8298,7 +8298,7 @@
       <c r="I3" s="1">
         <v>1852.66</v>
       </c>
-      <c r="K3" s="59" t="s">
+      <c r="K3" s="58" t="s">
         <v>154</v>
       </c>
     </row>
@@ -8331,7 +8331,7 @@
       <c r="I4" s="1">
         <v>1802.18</v>
       </c>
-      <c r="K4" s="66"/>
+      <c r="K4" s="59"/>
       <c r="L4" s="10"/>
     </row>
     <row r="5" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -8398,7 +8398,7 @@
         <v>1666.64</v>
       </c>
       <c r="K6" s="60"/>
-      <c r="M6" s="63" t="s">
+      <c r="M6" s="61" t="s">
         <v>154</v>
       </c>
     </row>
@@ -8431,7 +8431,7 @@
       <c r="I7" s="1">
         <v>1628.1</v>
       </c>
-      <c r="M7" s="64"/>
+      <c r="M7" s="62"/>
       <c r="N7" s="10"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -8460,7 +8460,7 @@
       <c r="I8">
         <v>1590.92</v>
       </c>
-      <c r="M8" s="62" t="s">
+      <c r="M8" s="63" t="s">
         <v>277</v>
       </c>
       <c r="O8" s="14"/>
@@ -8491,10 +8491,10 @@
       <c r="I9">
         <v>1544.14</v>
       </c>
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="58" t="s">
         <v>277</v>
       </c>
-      <c r="M9" s="62"/>
+      <c r="M9" s="63"/>
       <c r="O9" s="14"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -8523,7 +8523,7 @@
       <c r="I10">
         <v>1697.52</v>
       </c>
-      <c r="K10" s="66"/>
+      <c r="K10" s="59"/>
       <c r="L10" s="10"/>
       <c r="M10" s="14"/>
       <c r="O10" s="14"/>
@@ -8554,7 +8554,7 @@
       <c r="I11">
         <v>1643.86</v>
       </c>
-      <c r="K11" s="58" t="s">
+      <c r="K11" s="64" t="s">
         <v>275</v>
       </c>
       <c r="O11" s="14"/>
@@ -8585,8 +8585,8 @@
       <c r="I12">
         <v>1604.52</v>
       </c>
-      <c r="K12" s="58"/>
-      <c r="O12" s="62" t="s">
+      <c r="K12" s="64"/>
+      <c r="O12" s="63" t="s">
         <v>154</v>
       </c>
     </row>
@@ -8616,20 +8616,20 @@
       <c r="I13">
         <v>1465.8</v>
       </c>
-      <c r="O13" s="67"/>
+      <c r="O13" s="66"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H14" s="4"/>
-      <c r="O14" s="69" t="s">
+      <c r="O14" s="67" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H15" s="4"/>
-      <c r="K15" s="58" t="s">
+      <c r="K15" s="64" t="s">
         <v>147</v>
       </c>
-      <c r="O15" s="63"/>
+      <c r="O15" s="61"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H16" s="4"/>
@@ -8638,7 +8638,7 @@
       <c r="O16" s="14"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K17" s="59" t="s">
+      <c r="K17" s="58" t="s">
         <v>146</v>
       </c>
       <c r="M17" s="14"/>
@@ -8646,20 +8646,20 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="K18" s="59"/>
-      <c r="M18" s="62" t="s">
+      <c r="K18" s="58"/>
+      <c r="M18" s="63" t="s">
         <v>146</v>
       </c>
       <c r="O18" s="14"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="M19" s="67"/>
+      <c r="M19" s="66"/>
       <c r="N19" s="10"/>
       <c r="O19" s="14"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M20" s="69" t="s">
+      <c r="M20" s="67" t="s">
         <v>56</v>
       </c>
     </row>
@@ -8673,10 +8673,10 @@
       <c r="F21" s="16">
         <v>200</v>
       </c>
-      <c r="K21" s="59" t="s">
+      <c r="K21" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="M21" s="63"/>
+      <c r="M21" s="61"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
@@ -8691,7 +8691,7 @@
       <c r="F22" s="16">
         <v>100</v>
       </c>
-      <c r="K22" s="66"/>
+      <c r="K22" s="59"/>
       <c r="L22" s="10"/>
       <c r="M22" s="14"/>
     </row>
@@ -8706,7 +8706,7 @@
       <c r="F23" s="16">
         <v>30</v>
       </c>
-      <c r="K23" s="58" t="s">
+      <c r="K23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -8721,7 +8721,7 @@
       <c r="F24" s="16">
         <v>50</v>
       </c>
-      <c r="K24" s="58"/>
+      <c r="K24" s="64"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -8750,7 +8750,7 @@
       <c r="F26" s="16">
         <v>10</v>
       </c>
-      <c r="O26" s="58" t="s">
+      <c r="O26" s="64" t="s">
         <v>277</v>
       </c>
     </row>
@@ -8769,7 +8769,7 @@
       <c r="C28" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="O28" s="59" t="s">
+      <c r="O28" s="58" t="s">
         <v>146</v>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="O29" s="59"/>
+      <c r="O29" s="58"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
@@ -8788,11 +8788,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="K9:K10"/>
     <mergeCell ref="K23:K24"/>
     <mergeCell ref="O26:O27"/>
     <mergeCell ref="O28:O29"/>
@@ -8804,6 +8799,11 @@
     <mergeCell ref="M20:M21"/>
     <mergeCell ref="K21:K22"/>
     <mergeCell ref="K11:K12"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="K9:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8880,7 +8880,7 @@
       <c r="I2" s="1">
         <v>1401</v>
       </c>
-      <c r="K2" s="61" t="s">
+      <c r="K2" s="68" t="s">
         <v>216</v>
       </c>
     </row>
@@ -8913,8 +8913,8 @@
       <c r="I3" s="1">
         <v>1597</v>
       </c>
-      <c r="K3" s="61"/>
-      <c r="L3" s="59" t="s">
+      <c r="K3" s="68"/>
+      <c r="L3" s="58" t="s">
         <v>216</v>
       </c>
     </row>
@@ -8947,10 +8947,10 @@
       <c r="I4" s="1">
         <v>1324</v>
       </c>
-      <c r="K4" s="58" t="s">
+      <c r="K4" s="64" t="s">
         <v>219</v>
       </c>
-      <c r="L4" s="59"/>
+      <c r="L4" s="58"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -8981,7 +8981,7 @@
       <c r="I5" s="1">
         <v>1364</v>
       </c>
-      <c r="K5" s="58"/>
+      <c r="K5" s="64"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B6">
@@ -9039,7 +9039,7 @@
       <c r="I7">
         <v>1311</v>
       </c>
-      <c r="K7" s="58" t="s">
+      <c r="K7" s="64" t="s">
         <v>217</v>
       </c>
     </row>
@@ -9069,8 +9069,8 @@
       <c r="I8">
         <v>1200</v>
       </c>
-      <c r="K8" s="58"/>
-      <c r="L8" s="58" t="s">
+      <c r="K8" s="64"/>
+      <c r="L8" s="64" t="s">
         <v>217</v>
       </c>
     </row>
@@ -9100,13 +9100,13 @@
       <c r="I9">
         <v>985</v>
       </c>
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="58" t="s">
         <v>218</v>
       </c>
-      <c r="L9" s="58"/>
+      <c r="L9" s="64"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="K10" s="59"/>
+      <c r="K10" s="58"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L12" s="6" t="s">
@@ -9114,7 +9114,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="L13" s="58" t="s">
+      <c r="L13" s="64" t="s">
         <v>219</v>
       </c>
     </row>
@@ -9122,7 +9122,7 @@
       <c r="A14" t="s">
         <v>27</v>
       </c>
-      <c r="L14" s="58"/>
+      <c r="L14" s="64"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -9137,7 +9137,7 @@
       <c r="D15" t="s">
         <v>180</v>
       </c>
-      <c r="L15" s="59" t="s">
+      <c r="L15" s="58" t="s">
         <v>218</v>
       </c>
     </row>
@@ -9154,7 +9154,7 @@
       <c r="D16" t="s">
         <v>185</v>
       </c>
-      <c r="L16" s="59"/>
+      <c r="L16" s="58"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -14999,15 +14999,15 @@
         <v/>
       </c>
       <c r="U45" s="31">
-        <f t="shared" ref="U45:U68" si="5">SUM(F45:T45)</f>
+        <f>SUM(F45:T45)</f>
         <v>9</v>
       </c>
       <c r="V45" s="31">
-        <f t="shared" ref="V45:V68" si="6">SUM($F$27:$T$27)-SUMIFS($F$27:$T$27,$F45:$T45,"")</f>
+        <f t="shared" ref="V45:V68" si="5">SUM($F$27:$T$27)-SUMIFS($F$27:$T$27,$F45:$T45,"")</f>
         <v>14</v>
       </c>
       <c r="W45" s="31">
-        <f t="shared" ref="W45:W68" si="7">U45/V45</f>
+        <f t="shared" ref="W45:W68" si="6">U45/V45</f>
         <v>0.6428571428571429</v>
       </c>
       <c r="X45" s="29"/>
@@ -15106,15 +15106,15 @@
         <v>7</v>
       </c>
       <c r="U46" s="29">
+        <f t="shared" ref="U45:U68" si="7">SUM(F46:T46)</f>
+        <v>113</v>
+      </c>
+      <c r="V46" s="29">
         <f t="shared" si="5"/>
-        <v>113</v>
-      </c>
-      <c r="V46" s="29">
+        <v>203</v>
+      </c>
+      <c r="W46" s="30">
         <f t="shared" si="6"/>
-        <v>203</v>
-      </c>
-      <c r="W46" s="30">
-        <f t="shared" si="7"/>
         <v>0.55665024630541871</v>
       </c>
     </row>
@@ -15199,15 +15199,15 @@
         <v/>
       </c>
       <c r="U47" s="31">
+        <f t="shared" si="7"/>
+        <v>8</v>
+      </c>
+      <c r="V47" s="31">
         <f t="shared" si="5"/>
-        <v>8</v>
-      </c>
-      <c r="V47" s="31">
+        <v>14</v>
+      </c>
+      <c r="W47" s="31">
         <f t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="W47" s="31">
-        <f t="shared" si="7"/>
         <v>0.5714285714285714</v>
       </c>
       <c r="X47" s="29"/>
@@ -15293,15 +15293,15 @@
         <v>8</v>
       </c>
       <c r="U48" s="29">
+        <f t="shared" si="7"/>
+        <v>105</v>
+      </c>
+      <c r="V48" s="29">
         <f t="shared" si="5"/>
-        <v>105</v>
-      </c>
-      <c r="V48" s="29">
+        <v>203</v>
+      </c>
+      <c r="W48" s="30">
         <f t="shared" si="6"/>
-        <v>203</v>
-      </c>
-      <c r="W48" s="30">
-        <f t="shared" si="7"/>
         <v>0.51724137931034486</v>
       </c>
     </row>
@@ -15386,15 +15386,15 @@
         <v/>
       </c>
       <c r="U49" s="31">
+        <f t="shared" si="7"/>
+        <v>5</v>
+      </c>
+      <c r="V49" s="31">
         <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="V49" s="31">
+        <v>14</v>
+      </c>
+      <c r="W49" s="31">
         <f t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="W49" s="31">
-        <f t="shared" si="7"/>
         <v>0.35714285714285715</v>
       </c>
       <c r="X49" s="29"/>
@@ -15480,15 +15480,15 @@
         <v/>
       </c>
       <c r="U50" s="31">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="V50" s="31">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="V50" s="31">
+        <v>14</v>
+      </c>
+      <c r="W50" s="31">
         <f t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="W50" s="31">
-        <f t="shared" si="7"/>
         <v>0.2857142857142857</v>
       </c>
       <c r="X50" s="29"/>
@@ -15574,15 +15574,15 @@
         <v>7</v>
       </c>
       <c r="U51" s="29">
+        <f t="shared" si="7"/>
+        <v>103</v>
+      </c>
+      <c r="V51" s="29">
         <f t="shared" si="5"/>
-        <v>103</v>
-      </c>
-      <c r="V51" s="29">
+        <v>203</v>
+      </c>
+      <c r="W51" s="30">
         <f t="shared" si="6"/>
-        <v>203</v>
-      </c>
-      <c r="W51" s="30">
-        <f t="shared" si="7"/>
         <v>0.5073891625615764</v>
       </c>
     </row>
@@ -15664,15 +15664,15 @@
         <v/>
       </c>
       <c r="U52" s="31">
+        <f t="shared" si="7"/>
+        <v>9</v>
+      </c>
+      <c r="V52" s="31">
         <f t="shared" si="5"/>
-        <v>9</v>
-      </c>
-      <c r="V52" s="31">
+        <v>14</v>
+      </c>
+      <c r="W52" s="31">
         <f t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="W52" s="31">
-        <f t="shared" si="7"/>
         <v>0.6428571428571429</v>
       </c>
       <c r="X52" s="29"/>
@@ -15754,15 +15754,15 @@
         <v>5</v>
       </c>
       <c r="U53" s="29">
+        <f t="shared" si="7"/>
+        <v>100</v>
+      </c>
+      <c r="V53" s="29">
         <f t="shared" si="5"/>
-        <v>100</v>
-      </c>
-      <c r="V53" s="29">
+        <v>189</v>
+      </c>
+      <c r="W53" s="30">
         <f t="shared" si="6"/>
-        <v>189</v>
-      </c>
-      <c r="W53" s="30">
-        <f t="shared" si="7"/>
         <v>0.52910052910052907</v>
       </c>
     </row>
@@ -15844,15 +15844,15 @@
         <v/>
       </c>
       <c r="U54" s="34">
+        <f t="shared" si="7"/>
+        <v>74</v>
+      </c>
+      <c r="V54" s="34">
         <f t="shared" si="5"/>
-        <v>74</v>
-      </c>
-      <c r="V54" s="34">
+        <v>175</v>
+      </c>
+      <c r="W54" s="35">
         <f t="shared" si="6"/>
-        <v>175</v>
-      </c>
-      <c r="W54" s="35">
-        <f t="shared" si="7"/>
         <v>0.42285714285714288</v>
       </c>
     </row>
@@ -15933,15 +15933,15 @@
         <v>10</v>
       </c>
       <c r="U55" s="29">
+        <f t="shared" si="7"/>
+        <v>83</v>
+      </c>
+      <c r="V55" s="29">
         <f t="shared" si="5"/>
-        <v>83</v>
-      </c>
-      <c r="V55" s="29">
+        <v>189</v>
+      </c>
+      <c r="W55" s="30">
         <f t="shared" si="6"/>
-        <v>189</v>
-      </c>
-      <c r="W55" s="30">
-        <f t="shared" si="7"/>
         <v>0.43915343915343913</v>
       </c>
     </row>
@@ -16022,15 +16022,15 @@
         <v>7</v>
       </c>
       <c r="U56" s="29">
+        <f t="shared" si="7"/>
+        <v>87</v>
+      </c>
+      <c r="V56" s="29">
         <f t="shared" si="5"/>
-        <v>87</v>
-      </c>
-      <c r="V56" s="29">
+        <v>175</v>
+      </c>
+      <c r="W56" s="30">
         <f t="shared" si="6"/>
-        <v>175</v>
-      </c>
-      <c r="W56" s="30">
-        <f t="shared" si="7"/>
         <v>0.49714285714285716</v>
       </c>
     </row>
@@ -16112,15 +16112,15 @@
         <v/>
       </c>
       <c r="U57" s="31">
+        <f t="shared" si="7"/>
+        <v>5</v>
+      </c>
+      <c r="V57" s="31">
         <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="V57" s="31">
+        <v>14</v>
+      </c>
+      <c r="W57" s="31">
         <f t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="W57" s="31">
-        <f t="shared" si="7"/>
         <v>0.35714285714285715</v>
       </c>
       <c r="X57" s="29"/>
@@ -16203,15 +16203,15 @@
         <v/>
       </c>
       <c r="U58" s="31">
+        <f t="shared" si="7"/>
+        <v>23</v>
+      </c>
+      <c r="V58" s="31">
         <f t="shared" si="5"/>
-        <v>23</v>
-      </c>
-      <c r="V58" s="31">
+        <v>54</v>
+      </c>
+      <c r="W58" s="31">
         <f t="shared" si="6"/>
-        <v>54</v>
-      </c>
-      <c r="W58" s="31">
-        <f t="shared" si="7"/>
         <v>0.42592592592592593</v>
       </c>
       <c r="X58" s="29"/>
@@ -16294,15 +16294,15 @@
         <v/>
       </c>
       <c r="U59" s="31">
+        <f t="shared" si="7"/>
+        <v>3</v>
+      </c>
+      <c r="V59" s="31">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="V59" s="31">
+        <v>13</v>
+      </c>
+      <c r="W59" s="31">
         <f t="shared" si="6"/>
-        <v>13</v>
-      </c>
-      <c r="W59" s="31">
-        <f t="shared" si="7"/>
         <v>0.23076923076923078</v>
       </c>
       <c r="X59" s="29"/>
@@ -16384,15 +16384,15 @@
         <v>8</v>
       </c>
       <c r="U60" s="29">
+        <f t="shared" si="7"/>
+        <v>81</v>
+      </c>
+      <c r="V60" s="29">
         <f t="shared" si="5"/>
-        <v>81</v>
-      </c>
-      <c r="V60" s="29">
+        <v>161</v>
+      </c>
+      <c r="W60" s="30">
         <f t="shared" si="6"/>
-        <v>161</v>
-      </c>
-      <c r="W60" s="30">
-        <f t="shared" si="7"/>
         <v>0.50310559006211175</v>
       </c>
     </row>
@@ -16473,15 +16473,15 @@
         <v>5</v>
       </c>
       <c r="U61" s="29">
+        <f t="shared" si="7"/>
+        <v>76</v>
+      </c>
+      <c r="V61" s="29">
         <f t="shared" si="5"/>
-        <v>76</v>
-      </c>
-      <c r="V61" s="29">
+        <v>161</v>
+      </c>
+      <c r="W61" s="30">
         <f t="shared" si="6"/>
-        <v>161</v>
-      </c>
-      <c r="W61" s="30">
-        <f t="shared" si="7"/>
         <v>0.47204968944099379</v>
       </c>
     </row>
@@ -16563,15 +16563,15 @@
         <v/>
       </c>
       <c r="U62" s="31">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="V62" s="31">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="V62" s="31">
+        <v>13</v>
+      </c>
+      <c r="W62" s="31">
         <f t="shared" si="6"/>
-        <v>13</v>
-      </c>
-      <c r="W62" s="31">
-        <f t="shared" si="7"/>
         <v>0.30769230769230771</v>
       </c>
       <c r="X62" s="29"/>
@@ -16654,15 +16654,15 @@
         <v/>
       </c>
       <c r="U63" s="31">
+        <f t="shared" si="7"/>
+        <v>3</v>
+      </c>
+      <c r="V63" s="31">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="V63" s="31">
+        <v>13</v>
+      </c>
+      <c r="W63" s="31">
         <f t="shared" si="6"/>
-        <v>13</v>
-      </c>
-      <c r="W63" s="31">
-        <f t="shared" si="7"/>
         <v>0.23076923076923078</v>
       </c>
       <c r="X63" s="29"/>
@@ -16745,15 +16745,15 @@
         <v/>
       </c>
       <c r="U64" s="31">
+        <f t="shared" si="7"/>
+        <v>28</v>
+      </c>
+      <c r="V64" s="31">
         <f t="shared" si="5"/>
-        <v>28</v>
-      </c>
-      <c r="V64" s="31">
+        <v>52</v>
+      </c>
+      <c r="W64" s="31">
         <f t="shared" si="6"/>
-        <v>52</v>
-      </c>
-      <c r="W64" s="31">
-        <f t="shared" si="7"/>
         <v>0.53846153846153844</v>
       </c>
       <c r="X64" s="29"/>
@@ -16835,15 +16835,15 @@
         <v>11</v>
       </c>
       <c r="U65" s="29">
+        <f t="shared" si="7"/>
+        <v>69</v>
+      </c>
+      <c r="V65" s="29">
         <f t="shared" si="5"/>
-        <v>69</v>
-      </c>
-      <c r="V65" s="29">
+        <v>122</v>
+      </c>
+      <c r="W65" s="30">
         <f t="shared" si="6"/>
-        <v>122</v>
-      </c>
-      <c r="W65" s="30">
-        <f t="shared" si="7"/>
         <v>0.56557377049180324</v>
       </c>
     </row>
@@ -16925,15 +16925,15 @@
         <v/>
       </c>
       <c r="U66" s="31">
+        <f t="shared" si="7"/>
+        <v>23</v>
+      </c>
+      <c r="V66" s="31">
         <f t="shared" si="5"/>
-        <v>23</v>
-      </c>
-      <c r="V66" s="31">
+        <v>41</v>
+      </c>
+      <c r="W66" s="31">
         <f t="shared" si="6"/>
-        <v>41</v>
-      </c>
-      <c r="W66" s="31">
-        <f t="shared" si="7"/>
         <v>0.56097560975609762</v>
       </c>
       <c r="X66" s="29"/>
@@ -17015,15 +17015,15 @@
         <v>7</v>
       </c>
       <c r="U67" s="29">
+        <f>SUM(F67:T67)</f>
+        <v>23</v>
+      </c>
+      <c r="V67" s="29">
         <f t="shared" si="5"/>
-        <v>23</v>
-      </c>
-      <c r="V67" s="29">
+        <v>42</v>
+      </c>
+      <c r="W67" s="30">
         <f t="shared" si="6"/>
-        <v>42</v>
-      </c>
-      <c r="W67" s="30">
-        <f t="shared" si="7"/>
         <v>0.54761904761904767</v>
       </c>
     </row>
@@ -17036,15 +17036,15 @@
         <v>4</v>
       </c>
       <c r="U68" s="29">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
       <c r="V68" s="29">
+        <f>SUM($F$27:$T$27)-SUMIFS($F$27:$T$27,$F68:$T68,"")</f>
+        <v>14</v>
+      </c>
+      <c r="W68" s="30">
         <f t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="W68" s="30">
-        <f t="shared" si="7"/>
         <v>0.2857142857142857</v>
       </c>
       <c r="X68" s="29"/>
@@ -17290,7 +17290,7 @@
       <c r="I2" s="1">
         <v>1367</v>
       </c>
-      <c r="K2" s="61" t="s">
+      <c r="K2" s="68" t="s">
         <v>244</v>
       </c>
     </row>
@@ -17323,8 +17323,8 @@
       <c r="I3" s="1">
         <v>1409</v>
       </c>
-      <c r="K3" s="61"/>
-      <c r="L3" s="59" t="s">
+      <c r="K3" s="68"/>
+      <c r="L3" s="58" t="s">
         <v>244</v>
       </c>
     </row>
@@ -17357,10 +17357,10 @@
       <c r="I4" s="1">
         <v>1242</v>
       </c>
-      <c r="K4" s="58" t="s">
+      <c r="K4" s="64" t="s">
         <v>246</v>
       </c>
-      <c r="L4" s="59"/>
+      <c r="L4" s="58"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -17391,7 +17391,7 @@
       <c r="I5" s="1">
         <v>1280</v>
       </c>
-      <c r="K5" s="58"/>
+      <c r="K5" s="64"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B6">
@@ -17449,7 +17449,7 @@
       <c r="I7">
         <v>1055</v>
       </c>
-      <c r="K7" s="59" t="s">
+      <c r="K7" s="58" t="s">
         <v>245</v>
       </c>
     </row>
@@ -17479,8 +17479,8 @@
       <c r="I8">
         <v>1167</v>
       </c>
-      <c r="K8" s="59"/>
-      <c r="L8" s="58" t="s">
+      <c r="K8" s="58"/>
+      <c r="L8" s="64" t="s">
         <v>245</v>
       </c>
     </row>
@@ -17510,10 +17510,10 @@
       <c r="I9">
         <v>1162</v>
       </c>
-      <c r="K9" s="58" t="s">
+      <c r="K9" s="64" t="s">
         <v>247</v>
       </c>
-      <c r="L9" s="58"/>
+      <c r="L9" s="64"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B10">
@@ -17541,7 +17541,7 @@
       <c r="I10">
         <v>1086</v>
       </c>
-      <c r="K10" s="58"/>
+      <c r="K10" s="64"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B11">
@@ -17576,7 +17576,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="L13" s="59" t="s">
+      <c r="L13" s="58" t="s">
         <v>246</v>
       </c>
     </row>
@@ -17584,13 +17584,13 @@
       <c r="A14" t="s">
         <v>27</v>
       </c>
-      <c r="L14" s="59"/>
+      <c r="L14" s="58"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>173</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="L15" s="64" t="s">
         <v>247</v>
       </c>
     </row>
@@ -17598,7 +17598,7 @@
       <c r="A16" t="s">
         <v>28</v>
       </c>
-      <c r="L16" s="58"/>
+      <c r="L16" s="64"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -17708,7 +17708,7 @@
       <c r="I2" s="1">
         <v>1830.14</v>
       </c>
-      <c r="K2" s="58" t="s">
+      <c r="K2" s="64" t="s">
         <v>13</v>
       </c>
     </row>
@@ -17741,8 +17741,8 @@
       <c r="I3" s="1">
         <v>1705.42</v>
       </c>
-      <c r="K3" s="58"/>
-      <c r="L3" s="58" t="s">
+      <c r="K3" s="64"/>
+      <c r="L3" s="64" t="s">
         <v>259</v>
       </c>
     </row>
@@ -17775,10 +17775,10 @@
       <c r="I4" s="1">
         <v>1633.02</v>
       </c>
-      <c r="K4" s="59" t="s">
+      <c r="K4" s="58" t="s">
         <v>259</v>
       </c>
-      <c r="L4" s="58"/>
+      <c r="L4" s="64"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -17809,7 +17809,7 @@
       <c r="I5" s="1">
         <v>1611.72</v>
       </c>
-      <c r="K5" s="59"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B6">
@@ -17867,7 +17867,7 @@
       <c r="I7">
         <v>1547.34</v>
       </c>
-      <c r="K7" s="59" t="s">
+      <c r="K7" s="58" t="s">
         <v>258</v>
       </c>
     </row>
@@ -17897,8 +17897,8 @@
       <c r="I8">
         <v>1316.64</v>
       </c>
-      <c r="K8" s="59"/>
-      <c r="L8" s="59" t="s">
+      <c r="K8" s="58"/>
+      <c r="L8" s="58" t="s">
         <v>258</v>
       </c>
     </row>
@@ -17928,13 +17928,13 @@
       <c r="I9">
         <v>1320.34</v>
       </c>
-      <c r="K9" s="58" t="s">
+      <c r="K9" s="64" t="s">
         <v>260</v>
       </c>
-      <c r="L9" s="59"/>
+      <c r="L9" s="58"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="K10" s="58"/>
+      <c r="K10" s="64"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L12" s="6" t="s">
@@ -17942,7 +17942,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="L13" s="59" t="s">
+      <c r="L13" s="58" t="s">
         <v>13</v>
       </c>
     </row>
@@ -17953,7 +17953,7 @@
       <c r="B14" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="L14" s="59"/>
+      <c r="L14" s="58"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -17962,7 +17962,7 @@
       <c r="B15" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="L15" s="64" t="s">
         <v>260</v>
       </c>
     </row>
@@ -17973,7 +17973,7 @@
       <c r="B16" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="L16" s="58"/>
+      <c r="L16" s="64"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -18094,7 +18094,7 @@
       <c r="I2" s="1">
         <v>1636</v>
       </c>
-      <c r="K2" s="61" t="s">
+      <c r="K2" s="68" t="s">
         <v>7</v>
       </c>
     </row>
@@ -18127,8 +18127,8 @@
       <c r="I3" s="1">
         <v>1450</v>
       </c>
-      <c r="K3" s="61"/>
-      <c r="L3" s="61" t="s">
+      <c r="K3" s="68"/>
+      <c r="L3" s="68" t="s">
         <v>7</v>
       </c>
     </row>
@@ -18161,10 +18161,10 @@
       <c r="I4" s="1">
         <v>1333</v>
       </c>
-      <c r="K4" s="58" t="s">
+      <c r="K4" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="61"/>
+      <c r="L4" s="68"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -18195,7 +18195,7 @@
       <c r="I5" s="1">
         <v>1558</v>
       </c>
-      <c r="K5" s="58"/>
+      <c r="K5" s="64"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B6">
@@ -18253,7 +18253,7 @@
       <c r="I7">
         <v>1141</v>
       </c>
-      <c r="K7" s="58" t="s">
+      <c r="K7" s="64" t="s">
         <v>13</v>
       </c>
     </row>
@@ -18283,8 +18283,8 @@
       <c r="I8">
         <v>1174</v>
       </c>
-      <c r="K8" s="58"/>
-      <c r="L8" s="58" t="s">
+      <c r="K8" s="64"/>
+      <c r="L8" s="64" t="s">
         <v>9</v>
       </c>
     </row>
@@ -18314,13 +18314,13 @@
       <c r="I9">
         <v>1344</v>
       </c>
-      <c r="K9" s="59" t="s">
+      <c r="K9" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="L9" s="58"/>
+      <c r="L9" s="64"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="K10" s="59"/>
+      <c r="K10" s="58"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="L12" s="6" t="s">
@@ -18328,7 +18328,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="L13" s="58" t="s">
+      <c r="L13" s="64" t="s">
         <v>11</v>
       </c>
     </row>
@@ -18339,7 +18339,7 @@
       <c r="B14" t="s">
         <v>34</v>
       </c>
-      <c r="L14" s="58"/>
+      <c r="L14" s="64"/>
       <c r="M14" t="s">
         <v>11</v>
       </c>
@@ -18348,7 +18348,7 @@
       <c r="A15" t="s">
         <v>26</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="L15" s="64" t="s">
         <v>13</v>
       </c>
     </row>
@@ -18356,7 +18356,7 @@
       <c r="A16" t="s">
         <v>28</v>
       </c>
-      <c r="L16" s="58"/>
+      <c r="L16" s="64"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -18471,7 +18471,7 @@
       <c r="I2" s="1">
         <v>1511</v>
       </c>
-      <c r="K2" s="58" t="s">
+      <c r="K2" s="64" t="s">
         <v>9</v>
       </c>
     </row>
@@ -18504,8 +18504,8 @@
       <c r="I3" s="1">
         <v>1402</v>
       </c>
-      <c r="K3" s="58"/>
-      <c r="L3" s="59" t="s">
+      <c r="K3" s="64"/>
+      <c r="L3" s="58" t="s">
         <v>35</v>
       </c>
     </row>
@@ -18538,10 +18538,10 @@
       <c r="I4" s="1">
         <v>1297</v>
       </c>
-      <c r="K4" s="59" t="s">
+      <c r="K4" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="59"/>
+      <c r="L4" s="58"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -18572,7 +18572,7 @@
       <c r="I5" s="1">
         <v>1398</v>
       </c>
-      <c r="K5" s="59"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B6">
@@ -18630,7 +18630,7 @@
       <c r="I7">
         <v>1269</v>
       </c>
-      <c r="K7" s="59" t="s">
+      <c r="K7" s="58" t="s">
         <v>36</v>
       </c>
     </row>
@@ -18660,8 +18660,8 @@
       <c r="I8">
         <v>1254</v>
       </c>
-      <c r="K8" s="59"/>
-      <c r="L8" s="58" t="s">
+      <c r="K8" s="58"/>
+      <c r="L8" s="64" t="s">
         <v>9</v>
       </c>
     </row>
@@ -18691,10 +18691,10 @@
       <c r="I9">
         <v>1351</v>
       </c>
-      <c r="K9" s="58" t="s">
+      <c r="K9" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="L9" s="58"/>
+      <c r="L9" s="64"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B10">
@@ -18722,7 +18722,7 @@
       <c r="I10">
         <v>1294</v>
       </c>
-      <c r="K10" s="58"/>
+      <c r="K10" s="64"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B11">
@@ -18757,7 +18757,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="L13" s="59" t="s">
+      <c r="L13" s="58" t="s">
         <v>9</v>
       </c>
     </row>
@@ -18768,7 +18768,7 @@
       <c r="B14" t="s">
         <v>34</v>
       </c>
-      <c r="L14" s="59"/>
+      <c r="L14" s="58"/>
       <c r="M14" t="s">
         <v>9</v>
       </c>
@@ -18786,7 +18786,7 @@
       <c r="F15" s="15">
         <v>120</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="L15" s="64" t="s">
         <v>37</v>
       </c>
     </row>
@@ -18801,7 +18801,7 @@
       <c r="F16" s="15">
         <v>60</v>
       </c>
-      <c r="L16" s="58"/>
+      <c r="L16" s="64"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -18924,7 +18924,7 @@
       <c r="I2" s="1">
         <v>1844.5</v>
       </c>
-      <c r="K2" s="58" t="str">
+      <c r="K2" s="64" t="str">
         <f>C2</f>
         <v>#Hashtags</v>
       </c>
@@ -18958,8 +18958,8 @@
       <c r="I3" s="1">
         <v>2096.08</v>
       </c>
-      <c r="K3" s="58"/>
-      <c r="L3" s="59" t="s">
+      <c r="K3" s="64"/>
+      <c r="L3" s="58" t="s">
         <v>50</v>
       </c>
     </row>
@@ -18992,11 +18992,11 @@
       <c r="I4" s="1">
         <v>1811.46</v>
       </c>
-      <c r="K4" s="59" t="str">
+      <c r="K4" s="58" t="str">
         <f>C5</f>
         <v>Bologna Ponies</v>
       </c>
-      <c r="L4" s="59"/>
+      <c r="L4" s="58"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -19027,7 +19027,7 @@
       <c r="I5" s="1">
         <v>2048.5</v>
       </c>
-      <c r="K5" s="59"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B6">
@@ -19085,7 +19085,7 @@
       <c r="I7">
         <v>1774.8</v>
       </c>
-      <c r="K7" s="59" t="str">
+      <c r="K7" s="58" t="str">
         <f>C3</f>
         <v>The Timmies</v>
       </c>
@@ -19116,8 +19116,8 @@
       <c r="I8">
         <v>1793.28</v>
       </c>
-      <c r="K8" s="59"/>
-      <c r="L8" s="58" t="s">
+      <c r="K8" s="58"/>
+      <c r="L8" s="64" t="s">
         <v>51</v>
       </c>
     </row>
@@ -19147,11 +19147,11 @@
       <c r="I9">
         <v>1922.56</v>
       </c>
-      <c r="K9" s="58" t="str">
+      <c r="K9" s="64" t="str">
         <f>C4</f>
         <v>The dago</v>
       </c>
-      <c r="L9" s="58"/>
+      <c r="L9" s="64"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B10">
@@ -19179,7 +19179,7 @@
       <c r="I10">
         <v>1882.62</v>
       </c>
-      <c r="K10" s="58"/>
+      <c r="K10" s="64"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B11">
@@ -19214,7 +19214,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="L13" s="59" t="s">
+      <c r="L13" s="58" t="s">
         <v>7</v>
       </c>
     </row>
@@ -19225,7 +19225,7 @@
       <c r="B14" t="s">
         <v>34</v>
       </c>
-      <c r="L14" s="59"/>
+      <c r="L14" s="58"/>
       <c r="M14" t="s">
         <v>7</v>
       </c>
@@ -19243,7 +19243,7 @@
       <c r="F15" s="16">
         <v>120</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="L15" s="64" t="s">
         <v>52</v>
       </c>
     </row>
@@ -19257,7 +19257,7 @@
       <c r="F16" s="16">
         <v>60</v>
       </c>
-      <c r="L16" s="58"/>
+      <c r="L16" s="64"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -19403,7 +19403,7 @@
       <c r="J3" s="1">
         <v>1596.84</v>
       </c>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="58" t="s">
         <v>79</v>
       </c>
     </row>
@@ -19439,7 +19439,7 @@
       <c r="J4" s="1">
         <v>1481.24</v>
       </c>
-      <c r="L4" s="66"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -19512,7 +19512,7 @@
         <v>1635.62</v>
       </c>
       <c r="L6" s="60"/>
-      <c r="N6" s="62" t="s">
+      <c r="N6" s="63" t="s">
         <v>79</v>
       </c>
     </row>
@@ -19545,7 +19545,7 @@
       <c r="J7">
         <v>1508.98</v>
       </c>
-      <c r="N7" s="67"/>
+      <c r="N7" s="66"/>
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -19578,7 +19578,7 @@
       <c r="J8" s="10">
         <v>1388.18</v>
       </c>
-      <c r="N8" s="63" t="s">
+      <c r="N8" s="61" t="s">
         <v>51</v>
       </c>
       <c r="P8" s="14"/>
@@ -19587,10 +19587,10 @@
       <c r="A9" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="59" t="s">
+      <c r="L9" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="N9" s="63"/>
+      <c r="N9" s="61"/>
       <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -19624,7 +19624,7 @@
       <c r="J10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L10" s="66"/>
+      <c r="L10" s="59"/>
       <c r="M10" s="10"/>
       <c r="N10" s="14"/>
       <c r="P10" s="14"/>
@@ -19661,7 +19661,7 @@
       <c r="J11" s="1">
         <v>1673.14</v>
       </c>
-      <c r="L11" s="58" t="s">
+      <c r="L11" s="64" t="s">
         <v>61</v>
       </c>
       <c r="P11" s="14"/>
@@ -19698,8 +19698,8 @@
       <c r="J12" s="1">
         <v>1615.32</v>
       </c>
-      <c r="L12" s="58"/>
-      <c r="P12" s="63" t="s">
+      <c r="L12" s="64"/>
+      <c r="P12" s="61" t="s">
         <v>51</v>
       </c>
     </row>
@@ -19732,7 +19732,7 @@
       <c r="J13">
         <v>1539.26</v>
       </c>
-      <c r="P13" s="64"/>
+      <c r="P13" s="62"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B14">
@@ -19763,7 +19763,7 @@
       <c r="J14">
         <v>1336.24</v>
       </c>
-      <c r="P14" s="62" t="s">
+      <c r="P14" s="63" t="s">
         <v>70</v>
       </c>
     </row>
@@ -19796,10 +19796,10 @@
       <c r="J15">
         <v>1368.88</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="L15" s="64" t="s">
         <v>62</v>
       </c>
-      <c r="P15" s="62"/>
+      <c r="P15" s="63"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B16">
@@ -19835,7 +19835,7 @@
       <c r="P16" s="14"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L17" s="59" t="s">
+      <c r="L17" s="58" t="s">
         <v>70</v>
       </c>
       <c r="N17" s="14"/>
@@ -19843,20 +19843,20 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="L18" s="59"/>
-      <c r="N18" s="62" t="s">
+      <c r="L18" s="58"/>
+      <c r="N18" s="63" t="s">
         <v>70</v>
       </c>
       <c r="P18" s="14"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="N19" s="67"/>
+      <c r="N19" s="66"/>
       <c r="O19" s="10"/>
       <c r="P19" s="14"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N20" s="63" t="s">
+      <c r="N20" s="61" t="s">
         <v>60</v>
       </c>
     </row>
@@ -19870,10 +19870,10 @@
       <c r="F21" s="16">
         <v>120</v>
       </c>
-      <c r="L21" s="59" t="s">
+      <c r="L21" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="N21" s="63"/>
+      <c r="N21" s="61"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -19888,7 +19888,7 @@
       <c r="F22" s="16">
         <v>60</v>
       </c>
-      <c r="L22" s="66"/>
+      <c r="L22" s="59"/>
       <c r="M22" s="10"/>
       <c r="N22" s="14"/>
     </row>
@@ -19902,7 +19902,7 @@
       <c r="F23" s="16">
         <v>20</v>
       </c>
-      <c r="L23" s="58" t="s">
+      <c r="L23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -19910,7 +19910,7 @@
       <c r="A24" t="s">
         <v>28</v>
       </c>
-      <c r="L24" s="58"/>
+      <c r="L24" s="64"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -19924,7 +19924,7 @@
       <c r="A26" t="s">
         <v>30</v>
       </c>
-      <c r="P26" s="58" t="s">
+      <c r="P26" s="64" t="s">
         <v>79</v>
       </c>
     </row>
@@ -19938,7 +19938,7 @@
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="P28" s="59" t="s">
+      <c r="P28" s="58" t="s">
         <v>60</v>
       </c>
     </row>
@@ -19946,13 +19946,19 @@
       <c r="A29" t="s">
         <v>49</v>
       </c>
-      <c r="P29" s="59"/>
+      <c r="P29" s="58"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C11:J16">
     <sortCondition descending="1" ref="H11:H16"/>
   </sortState>
   <mergeCells count="16">
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="P12:P13"/>
+    <mergeCell ref="P28:P29"/>
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="L21:L22"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="N8:N9"/>
@@ -19963,12 +19969,6 @@
     <mergeCell ref="L11:L12"/>
     <mergeCell ref="L15:L16"/>
     <mergeCell ref="L17:L18"/>
-    <mergeCell ref="P14:P15"/>
-    <mergeCell ref="P12:P13"/>
-    <mergeCell ref="P28:P29"/>
-    <mergeCell ref="P26:P27"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="L21:L22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -20069,7 +20069,7 @@
       <c r="J3" s="1">
         <v>1732.22</v>
       </c>
-      <c r="L3" s="59" t="s">
+      <c r="L3" s="58" t="s">
         <v>86</v>
       </c>
     </row>
@@ -20105,7 +20105,7 @@
       <c r="J4" s="1">
         <v>1639.06</v>
       </c>
-      <c r="L4" s="66"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -20178,7 +20178,7 @@
         <v>1643.26</v>
       </c>
       <c r="L6" s="60"/>
-      <c r="N6" s="62" t="s">
+      <c r="N6" s="63" t="s">
         <v>86</v>
       </c>
     </row>
@@ -20211,7 +20211,7 @@
       <c r="J7">
         <v>1588.24</v>
       </c>
-      <c r="N7" s="67"/>
+      <c r="N7" s="66"/>
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -20244,7 +20244,7 @@
       <c r="J8" s="10">
         <v>1475.86</v>
       </c>
-      <c r="N8" s="63" t="s">
+      <c r="N8" s="61" t="s">
         <v>89</v>
       </c>
       <c r="P8" s="14"/>
@@ -20253,10 +20253,10 @@
       <c r="A9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L9" s="58" t="s">
+      <c r="L9" s="64" t="s">
         <v>73</v>
       </c>
-      <c r="N9" s="63"/>
+      <c r="N9" s="61"/>
       <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -20327,7 +20327,7 @@
       <c r="J11" s="1">
         <v>1625.18</v>
       </c>
-      <c r="L11" s="59" t="s">
+      <c r="L11" s="58" t="s">
         <v>89</v>
       </c>
       <c r="P11" s="14"/>
@@ -20364,8 +20364,8 @@
       <c r="J12" s="1">
         <v>1578.96</v>
       </c>
-      <c r="L12" s="59"/>
-      <c r="P12" s="63" t="s">
+      <c r="L12" s="58"/>
+      <c r="P12" s="61" t="s">
         <v>86</v>
       </c>
     </row>
@@ -20398,7 +20398,7 @@
       <c r="J13">
         <v>1497.04</v>
       </c>
-      <c r="P13" s="64"/>
+      <c r="P13" s="62"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B14">
@@ -20429,7 +20429,7 @@
       <c r="J14">
         <v>1303.76</v>
       </c>
-      <c r="P14" s="62" t="s">
+      <c r="P14" s="63" t="s">
         <v>88</v>
       </c>
     </row>
@@ -20462,10 +20462,10 @@
       <c r="J15">
         <v>1504.64</v>
       </c>
-      <c r="L15" s="58" t="s">
+      <c r="L15" s="64" t="s">
         <v>87</v>
       </c>
-      <c r="P15" s="62"/>
+      <c r="P15" s="63"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B16">
@@ -20501,7 +20501,7 @@
       <c r="P16" s="14"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L17" s="59" t="s">
+      <c r="L17" s="58" t="s">
         <v>72</v>
       </c>
       <c r="N17" s="14"/>
@@ -20509,20 +20509,20 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H18" s="4"/>
-      <c r="L18" s="59"/>
-      <c r="N18" s="62" t="s">
+      <c r="L18" s="58"/>
+      <c r="N18" s="63" t="s">
         <v>72</v>
       </c>
       <c r="P18" s="14"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="H19" s="4"/>
-      <c r="N19" s="67"/>
+      <c r="N19" s="66"/>
       <c r="O19" s="10"/>
       <c r="P19" s="14"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="N20" s="63" t="s">
+      <c r="N20" s="61" t="s">
         <v>88</v>
       </c>
     </row>
@@ -20536,10 +20536,10 @@
       <c r="F21" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="L21" s="59" t="s">
+      <c r="L21" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="N21" s="63"/>
+      <c r="N21" s="61"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -20554,7 +20554,7 @@
       <c r="F22" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="L22" s="66"/>
+      <c r="L22" s="59"/>
       <c r="M22" s="10"/>
       <c r="N22" s="14"/>
     </row>
@@ -20568,7 +20568,7 @@
       <c r="F23" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="L23" s="58" t="s">
+      <c r="L23" s="64" t="s">
         <v>80</v>
       </c>
     </row>
@@ -20580,7 +20580,7 @@
         <v>112</v>
       </c>
       <c r="F24" s="16"/>
-      <c r="L24" s="58"/>
+      <c r="L24" s="64"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -20595,7 +20595,7 @@
       <c r="A26" t="s">
         <v>30</v>
       </c>
-      <c r="P26" s="59" t="s">
+      <c r="P26" s="58" t="s">
         <v>89</v>
       </c>
     </row>
@@ -20603,13 +20603,13 @@
       <c r="A27" t="s">
         <v>83</v>
       </c>
-      <c r="P27" s="66"/>
+      <c r="P27" s="59"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="P28" s="58" t="s">
+      <c r="P28" s="64" t="s">
         <v>72</v>
       </c>
     </row>
@@ -20617,18 +20617,13 @@
       <c r="A29" t="s">
         <v>49</v>
       </c>
-      <c r="P29" s="58"/>
+      <c r="P29" s="64"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C11:J16">
     <sortCondition descending="1" ref="H11:H16"/>
   </sortState>
   <mergeCells count="16">
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="L9:L10"/>
     <mergeCell ref="L23:L24"/>
     <mergeCell ref="P26:P27"/>
     <mergeCell ref="P28:P29"/>
@@ -20640,6 +20635,11 @@
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="L21:L22"/>
     <mergeCell ref="L11:L12"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="L9:L10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
18May26 - PRO - updated GoodellBot to use GIPHY instead of tenor, notes, etc
</commit_message>
<xml_diff>
--- a/TeamFriends_History.xlsx
+++ b/TeamFriends_History.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Sites\TeamFriendsFantasy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B123BD0-A986-46A0-B697-486E12ACAD14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{673EDD28-98A6-42F8-96DA-A4DB570A68B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="677" firstSheet="1" activeTab="19" xr2:uid="{960D14EB-F112-4860-840A-1E6B67EAFFB3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="677" activeTab="8" xr2:uid="{960D14EB-F112-4860-840A-1E6B67EAFFB3}"/>
   </bookViews>
   <sheets>
     <sheet name="2005" sheetId="16" r:id="rId1"/>
@@ -12486,9 +12486,9 @@
         <f>_xlfn.XLOOKUP($A17,'2014'!$D$3:$D$16,'2014'!$B$3:$B$16,"")</f>
         <v>6</v>
       </c>
-      <c r="J17" t="str">
+      <c r="J17">
         <f>_xlfn.XLOOKUP($A17,'2015'!$D$3:$D$16,'2015'!$B$3:$B$16,"")</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="K17" t="str">
         <f>_xlfn.XLOOKUP($A17,'2016'!$D$3:$D$16,'2016'!$B$3:$B$16,"")</f>
@@ -12565,9 +12565,9 @@
         <f>_xlfn.XLOOKUP($A17,'2014'!$D$3:$D$16,'2014'!$A$3:$A$16,"x")</f>
         <v>0</v>
       </c>
-      <c r="AG17" s="31" t="str">
+      <c r="AG17" s="31">
         <f>_xlfn.XLOOKUP($A17,'2015'!$D$3:$D$16,'2015'!$A$3:$A$16,"x")</f>
-        <v>x</v>
+        <v>0</v>
       </c>
       <c r="AH17" s="31" t="str">
         <f>_xlfn.XLOOKUP($A17,'2016'!$D$3:$D$16,'2016'!$A$3:$A$16,"x")</f>
@@ -13038,9 +13038,9 @@
         <f>_xlfn.XLOOKUP($A20,'2014'!$D$3:$D$16,'2014'!$B$3:$B$16,"")</f>
         <v/>
       </c>
-      <c r="J20">
+      <c r="J20" t="str">
         <f>_xlfn.XLOOKUP($A20,'2015'!$D$3:$D$16,'2015'!$B$3:$B$16,"")</f>
-        <v>11</v>
+        <v/>
       </c>
       <c r="K20" t="str">
         <f>_xlfn.XLOOKUP($A20,'2016'!$D$3:$D$16,'2016'!$B$3:$B$16,"")</f>
@@ -13117,9 +13117,9 @@
         <f>_xlfn.XLOOKUP($A20,'2014'!$D$3:$D$16,'2014'!$A$3:$A$16,"x")</f>
         <v>x</v>
       </c>
-      <c r="AG20" s="31">
+      <c r="AG20" s="31" t="str">
         <f>_xlfn.XLOOKUP($A20,'2015'!$D$3:$D$16,'2015'!$A$3:$A$16,"x")</f>
-        <v>0</v>
+        <v>x</v>
       </c>
       <c r="AH20" s="31" t="str">
         <f>_xlfn.XLOOKUP($A20,'2016'!$D$3:$D$16,'2016'!$A$3:$A$16,"x")</f>
@@ -13161,9 +13161,9 @@
         <f>_xlfn.XLOOKUP($A20,'2025'!$D$2:$D$13,'2025'!$A$2:$A$13,"x")</f>
         <v>x</v>
       </c>
-      <c r="AR20" s="32">
+      <c r="AR20" s="32" t="e">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="AS20" s="31">
         <f t="shared" si="1"/>
@@ -13177,13 +13177,13 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AV20" s="32">
+      <c r="AV20" s="32" t="e">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AW20" s="51">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AW20" s="51" t="e">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="21" spans="1:49" x14ac:dyDescent="0.25">
@@ -15003,7 +15003,7 @@
         <v>9</v>
       </c>
       <c r="V45" s="31">
-        <f t="shared" ref="V45:V68" si="5">SUM($F$27:$T$27)-SUMIFS($F$27:$T$27,$F45:$T45,"")</f>
+        <f t="shared" ref="V45:V67" si="5">SUM($F$27:$T$27)-SUMIFS($F$27:$T$27,$F45:$T45,"")</f>
         <v>14</v>
       </c>
       <c r="W45" s="31">
@@ -15106,7 +15106,7 @@
         <v>7</v>
       </c>
       <c r="U46" s="29">
-        <f t="shared" ref="U45:U68" si="7">SUM(F46:T46)</f>
+        <f t="shared" ref="U46:U68" si="7">SUM(F46:T46)</f>
         <v>113</v>
       </c>
       <c r="V46" s="29">
@@ -16249,9 +16249,9 @@
         <f>_xlfn.XLOOKUP($A59,'2014'!$D$3:$D$16,'2014'!$E$3:$E$16,"")</f>
         <v>3</v>
       </c>
-      <c r="J59" s="31" t="str">
+      <c r="J59" s="31">
         <f>_xlfn.XLOOKUP($A59,'2015'!$D$3:$D$16,'2015'!$E$3:$E$16,"")</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="K59" s="31" t="str">
         <f>_xlfn.XLOOKUP($A59,'2016'!$D$3:$D$16,'2016'!$E$3:$E$16,"")</f>
@@ -16295,15 +16295,15 @@
       </c>
       <c r="U59" s="31">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="V59" s="31">
         <f t="shared" si="5"/>
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="W59" s="31">
         <f t="shared" si="6"/>
-        <v>0.23076923076923078</v>
+        <v>0.26923076923076922</v>
       </c>
       <c r="X59" s="29"/>
     </row>
@@ -16518,9 +16518,9 @@
         <f>_xlfn.XLOOKUP($A62,'2014'!$D$3:$D$16,'2014'!$E$3:$E$16,"")</f>
         <v/>
       </c>
-      <c r="J62" s="31">
+      <c r="J62" s="31" t="str">
         <f>_xlfn.XLOOKUP($A62,'2015'!$D$3:$D$16,'2015'!$E$3:$E$16,"")</f>
-        <v>4</v>
+        <v/>
       </c>
       <c r="K62" s="31" t="str">
         <f>_xlfn.XLOOKUP($A62,'2016'!$D$3:$D$16,'2016'!$E$3:$E$16,"")</f>
@@ -16564,15 +16564,15 @@
       </c>
       <c r="U62" s="31">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V62" s="31">
         <f t="shared" si="5"/>
-        <v>13</v>
-      </c>
-      <c r="W62" s="31">
+        <v>0</v>
+      </c>
+      <c r="W62" s="31" t="e">
         <f t="shared" si="6"/>
-        <v>0.30769230769230771</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="X62" s="29"/>
     </row>
@@ -20441,7 +20441,7 @@
         <v>64</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E15">
         <v>4</v>

</xml_diff>